<commit_message>
Stage 8 review fixes: B-029
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2026/BW26_0368/Run_sheets/BW26_0368_RUN04.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2026/BW26_0368/Run_sheets/BW26_0368_RUN04.xlsx
@@ -184,7 +184,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Recovery on the 2 h read is low for two compounds. Check the recovery column before anyone quotes the free fraction.</t>
+        <t>Use the recorded unbound percentage; subtracting the rounded bound value may give a different last digit. Retain the recovery column with each result.</t>
       </text>
     </comment>
   </commentList>
@@ -492,7 +492,8 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BW26_0368 run sheet 04: microsomal stability and RED PPB (INTERIM)</t>
+          <t>Brindlewythe Biosciences Ltd, a Tarnovell company
+BW26_0368 run sheet 04: microsomal stability and RED PPB (INTERIM)</t>
         </is>
       </c>
     </row>
@@ -559,7 +560,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Compounds on run</t>
+          <t>Compounds on project</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -581,7 +582,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Runs</t>
+          <t>Study start / interim</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -631,7 +632,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Batch</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -663,7 +664,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Compound set A</t>
+          <t>Sample card reconciliation</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
@@ -673,7 +674,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Compound set B</t>
+          <t>Remaining result rows</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
@@ -716,7 +717,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Human and rat CLint and half-life. Repeat pending for the compounds flagged in the interim summary.</t>
+          <t>Human and rat CLint and half-life; partial interim results. Verapamil and diltiazem controls were within historical range for the reported runs. The final stability repeat awaits the delayed reference-control shipment.</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1032,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>First set of compounds read and reconciled. Remaining compounds are queued behind the control shipment.</t>
+          <t>Partial interim binding results, RED, 4 h, 37 °C. Recovery has been reconciled for the reported rows; remaining rows are in progress. Warfarin is the binding control.</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1241,8 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Interim summary</t>
+          <t>Brindlewythe Biosciences Ltd, a Tarnovell company
+Interim summary</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1254,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Interim: binding complete for the first set; stability repeat pending.</t>
+          <t>Interim: binding recovery reconciled for reported rows; stability repeat and remaining result rows pending.</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1289,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Stability repeat after the control shipment; binding for the remaining compounds; biology memo review.</t>
+          <t>Final stability repeat after reference-control shipment; complete remaining result rows. No final conclusions yet.</t>
         </is>
       </c>
     </row>

</xml_diff>